<commit_message>
Updated the game data
</commit_message>
<xml_diff>
--- a/public/gameData/quiz-data.xlsx
+++ b/public/gameData/quiz-data.xlsx
@@ -5,20 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charlie\Desktop\gridReveal\public\gameData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charlie\Desktop\web-games\gridReveal\public\gameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A9BDD4-5B8E-43DD-AD48-CCC421578D2B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C999D93-2E0D-4830-AF85-1C902E1697EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="g1-general-knowledge" sheetId="6" r:id="rId1"/>
-    <sheet name="g3-system-unit" sheetId="7" r:id="rId2"/>
-    <sheet name="g5-computer-network" sheetId="8" r:id="rId3"/>
-    <sheet name="g2-parts-of-a-computer" sheetId="9" r:id="rId4"/>
-    <sheet name="kg-computer-parts" sheetId="10" r:id="rId5"/>
-    <sheet name="g5-types-of-network" sheetId="11" r:id="rId6"/>
+    <sheet name="g2-color-mixing" sheetId="12" r:id="rId1"/>
+    <sheet name="g1-general-knowledge" sheetId="6" r:id="rId2"/>
+    <sheet name="g3-system-unit" sheetId="7" r:id="rId3"/>
+    <sheet name="g5-computer-network" sheetId="8" r:id="rId4"/>
+    <sheet name="g2-parts-of-a-computer" sheetId="9" r:id="rId5"/>
+    <sheet name="kg-computer-parts" sheetId="10" r:id="rId6"/>
+    <sheet name="g5-types-of-network" sheetId="11" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="241">
   <si>
     <t>Questions</t>
   </si>
@@ -630,6 +631,129 @@
   </si>
   <si>
     <t>Personal Area Network</t>
+  </si>
+  <si>
+    <t>Color Mixing</t>
+  </si>
+  <si>
+    <t>https://justpaint.org/wp-content/uploads/2015/06/2a1.jpg</t>
+  </si>
+  <si>
+    <t>To learn about color mixing</t>
+  </si>
+  <si>
+    <t>Yellow + Red = ____________.</t>
+  </si>
+  <si>
+    <t>https://media.baamboozle.com/uploads/images/795443/3e13b13e-7363-42d3-9654-0b7dd87c13c0.jpeg</t>
+  </si>
+  <si>
+    <t>Red + Blue = ____________.</t>
+  </si>
+  <si>
+    <t>Purple</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcSA0avufhAE-GhtSr-melhdRd0Gyqx6vHax-SBCBH-7Jg&amp;s=10</t>
+  </si>
+  <si>
+    <t>Blue + Yellow = ____________.</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcR275EN_zLGZXOYnGUCLnaR3TEN_En_6DGNz586_sX21w&amp;s=10</t>
+  </si>
+  <si>
+    <t>Red + White = ____________.</t>
+  </si>
+  <si>
+    <t>Pink</t>
+  </si>
+  <si>
+    <t>https://i5.walmartimages.com/seo/Valentine-s-Day-8-Red-White-Teddy-Bear-Plush-by-Way-To-Celebrate_66d89fb6-af26-498f-9217-bec98b8a9f1f.81edabb2c88900bd55f5dde963cd3c5e.jpeg</t>
+  </si>
+  <si>
+    <t>Black + White = ____________.</t>
+  </si>
+  <si>
+    <t>Gray</t>
+  </si>
+  <si>
+    <t>https://img.magnific.com/free-vector/abstract-background-with-black-white-warped-pattern_1048-20191.jpg?semt=ais_hybrid&amp;w=740&amp;q=80</t>
+  </si>
+  <si>
+    <t>Blue + White = ____________.</t>
+  </si>
+  <si>
+    <t>Light Blue</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQwxh_WUKM_-r10l9trLh54ScEAT_Ff5GlDGNy-CvLv5g&amp;s=10</t>
+  </si>
+  <si>
+    <t>Red + Yellow + Blue = ____________.</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcSPEOM5T6M1cnjnunTRdLA_Qpp32HOVr--HE503b-RTMA&amp;s=10</t>
+  </si>
+  <si>
+    <t>What color do you get by mixing Yellow and Blue?</t>
+  </si>
+  <si>
+    <t>What color do you get by mixing Red and Blue?</t>
+  </si>
+  <si>
+    <t>What color do you get by mixing Red and Yellow?</t>
+  </si>
+  <si>
+    <t>Which two colors make Green?</t>
+  </si>
+  <si>
+    <t>Blue + Yellow</t>
+  </si>
+  <si>
+    <t>Which two colors make Orange?</t>
+  </si>
+  <si>
+    <t>Red + Yellow</t>
+  </si>
+  <si>
+    <t>Which two colors make Purple?</t>
+  </si>
+  <si>
+    <t>Red + Blue</t>
+  </si>
+  <si>
+    <t>Which color is made by mixing Red and White?</t>
+  </si>
+  <si>
+    <t>Which color is made by mixing Black and White?</t>
+  </si>
+  <si>
+    <t>What color do you get by adding White to Blue?</t>
+  </si>
+  <si>
+    <t>What color do you get by adding White to Red?</t>
+  </si>
+  <si>
+    <t>Green is made by mixing ____________ and ____________.</t>
+  </si>
+  <si>
+    <t>Blue, Yellow</t>
+  </si>
+  <si>
+    <t>Orange is made by mixing ____________ and ____________.</t>
+  </si>
+  <si>
+    <t>Red, Yellow</t>
+  </si>
+  <si>
+    <t>Purple is made by mixing ____________ and ____________.</t>
+  </si>
+  <si>
+    <t>Red, Blue</t>
   </si>
 </sst>
 </file>
@@ -1054,6 +1178,854 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51A97C99-3E7F-46D4-9C42-6A91E0C55022}">
+  <dimension ref="A1:E91"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44" style="2" customWidth="1"/>
+    <col min="2" max="2" width="44" style="10" customWidth="1"/>
+    <col min="3" max="3" width="44" style="2" customWidth="1"/>
+    <col min="4" max="4" width="48.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+    </row>
+    <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="10">
+        <v>15</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" s="10">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="10">
+        <v>15</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="C12" s="10">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" s="10">
+        <v>15</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="C14" s="10">
+        <v>15</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="C15" s="10">
+        <v>20</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="10">
+        <v>20</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="C17" s="10">
+        <v>20</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="10">
+        <v>20</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="C19" s="10">
+        <v>20</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="C20" s="10">
+        <v>20</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="C21" s="10">
+        <v>20</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="C22" s="10">
+        <v>20</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="C23" s="10">
+        <v>20</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="C24" s="10">
+        <v>20</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="C25" s="10">
+        <v>20</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C26" s="10">
+        <v>25</v>
+      </c>
+      <c r="D26" s="1"/>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="C27" s="10">
+        <v>25</v>
+      </c>
+      <c r="D27" s="1"/>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="C28" s="10">
+        <v>25</v>
+      </c>
+      <c r="D28" s="1"/>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="2"/>
+    </row>
+    <row r="45" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="2"/>
+    </row>
+    <row r="57" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="2"/>
+    </row>
+    <row r="58" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="60" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="2"/>
+    </row>
+    <row r="63" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="2"/>
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="2"/>
+    </row>
+    <row r="64" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="2"/>
+    </row>
+    <row r="65" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="2"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="2"/>
+    </row>
+    <row r="66" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="2"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="2"/>
+    </row>
+    <row r="67" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="2"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="2"/>
+    </row>
+    <row r="68" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="2"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="2"/>
+    </row>
+    <row r="69" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="2"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="2"/>
+    </row>
+    <row r="70" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2"/>
+      <c r="B70" s="10"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="2"/>
+    </row>
+    <row r="71" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="2"/>
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="2"/>
+    </row>
+    <row r="72" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2"/>
+      <c r="B72" s="10"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="2"/>
+    </row>
+    <row r="73" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="2"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="2"/>
+    </row>
+    <row r="74" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="2"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="2"/>
+    </row>
+    <row r="75" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="2"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="2"/>
+    </row>
+    <row r="76" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="2"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="2"/>
+    </row>
+    <row r="77" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="2"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="2"/>
+    </row>
+    <row r="78" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2"/>
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="2"/>
+    </row>
+    <row r="79" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="2"/>
+    </row>
+    <row r="80" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="2"/>
+      <c r="B80" s="10"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="2"/>
+    </row>
+    <row r="81" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="2"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="2"/>
+    </row>
+    <row r="82" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="2"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="2"/>
+    </row>
+    <row r="83" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="2"/>
+      <c r="B83" s="10"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="2"/>
+    </row>
+    <row r="84" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="2"/>
+      <c r="B84" s="10"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="2"/>
+    </row>
+    <row r="85" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="2"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="2"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="2"/>
+    </row>
+    <row r="86" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="2"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="5"/>
+      <c r="E86" s="2"/>
+    </row>
+    <row r="87" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="2"/>
+      <c r="B87" s="10"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="2"/>
+    </row>
+    <row r="88" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="2"/>
+      <c r="B88" s="10"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="5"/>
+      <c r="E88" s="2"/>
+    </row>
+    <row r="89" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="2"/>
+      <c r="B89" s="10"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="2"/>
+    </row>
+    <row r="90" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="2"/>
+      <c r="B90" s="10"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="2"/>
+    </row>
+    <row r="91" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="2"/>
+      <c r="B91" s="10"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3" xr:uid="{1333C3A6-160B-4E52-A5C0-C41B8CAB389C}">
+      <formula1>"KG, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5" xr:uid="{088CF47A-38AD-4DD0-9F67-3811FE96DA17}">
+      <formula1>"English, Computer, Science, Math, Geography, History, General Knowledge, Social Studies, Life Skills"</formula1>
+    </dataValidation>
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{BAF3AA5D-9B29-4633-94F2-2AB3EB27B028}">
+      <formula1>3</formula1>
+      <formula2>25</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9:C249" xr:uid="{6BF6D43C-45CA-484C-A0B6-72F4F3A63360}">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B76B5DC4-6C72-4A29-A7BE-2FD0D1E3D641}">
   <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1941,7 +2913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{444B2F6E-3FF4-4A0B-8E9C-C725ED3F5542}">
   <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2758,7 +3730,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7C45BDA-9308-4B5D-A47F-02AF42687C21}">
   <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3548,7 +4520,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9263046-FE36-46C5-AE2F-052E66BED452}">
   <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4383,7 +5355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16BE6E6A-CFE5-4EEB-AB25-4CDF6513BCB5}">
   <dimension ref="A1:E83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5122,7 +6094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF5EDB16-6A22-405A-8C30-5681553FE3DB}">
   <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>